<commit_message>
configuracion de nuevo step, metrica nueva de resultados
</commit_message>
<xml_diff>
--- a/data/database/dimensions.xlsx
+++ b/data/database/dimensions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -672,6 +672,84 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pregunta</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-03-02 11:02:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Habilidad</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-03-02 15:19:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>13</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Eje Temático</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-03-02 15:19:02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nuevas métricas, carga de valores
</commit_message>
<xml_diff>
--- a/data/database/dimensions.xlsx
+++ b/data/database/dimensions.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -750,6 +754,126 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Hito</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" s="2" t="n">
+        <v>46093.54063716435</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Nivel</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
+        <v>46093.54063716435</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>16</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>N Pregunta</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>46093.54595423849</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>17</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>N OA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>46093.54595423849</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>18</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Indicador</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>46093.54595423849</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: ensure achievement_levels is an array in NewIndicatorDrawer component
</commit_message>
<xml_diff>
--- a/data/database/dimensions.xlsx
+++ b/data/database/dimensions.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -930,6 +930,32 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>21</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:48:23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>